<commit_message>
Support display permissions on user create + Excel import
הרשאות התצוגה (הצגת רכישות בחיפוש / הצגת מסך "הרכישות שלי") היו זמינות
רק בעריכת משתמש. כעת זמינות גם:
- בטופס יצירת משתמש (שני צ'קבוקסים, ברירת מחדל מסומן)
- בטעינת משתמשים מאקסל (עמודות רשות "הצגת רכישות בחיפוש"/"הצגת הרכישות שלי", כן/לא)
התבנית עודכנה בהתאם.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/users-template.xlsx
+++ b/public/templates/users-template.xlsx
@@ -397,7 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G3"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,44 +424,62 @@
       <c r="E1" t="str">
         <v>תפקיד</v>
       </c>
+      <c r="F1" t="str">
+        <v>הצגת רכישות בחיפוש</v>
+      </c>
+      <c r="G1" t="str">
+        <v>הצגת הרכישות שלי</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>ישראל ישראלי</v>
       </c>
       <c r="B2" t="str">
-        <v>user@example.com</v>
+        <v>israel@example.com</v>
       </c>
       <c r="C2" t="str">
-        <v>050-0000000</v>
+        <v>0501234567</v>
       </c>
       <c r="D2" t="str">
-        <v>משק הירדן</v>
+        <v>משק לדוגמה</v>
       </c>
       <c r="E2" t="str">
         <v>משתמש רגיל</v>
+      </c>
+      <c r="F2" t="str">
+        <v>כן</v>
+      </c>
+      <c r="G2" t="str">
+        <v>כן</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>מנהל לדוגמה</v>
+        <v>דנה כהן</v>
       </c>
       <c r="B3" t="str">
-        <v>admin@example.com</v>
+        <v>dana@example.com</v>
       </c>
       <c r="C3" t="str">
-        <v>050-1111111</v>
+        <v>0529876543</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>משק לדוגמה</v>
       </c>
       <c r="E3" t="str">
-        <v>מנהל</v>
+        <v>משתמש רגיל</v>
+      </c>
+      <c r="F3" t="str">
+        <v>כן</v>
+      </c>
+      <c r="G3" t="str">
+        <v>לא</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>